<commit_message>
fix: promotion per-class sequences + root route for uptime monitors
</commit_message>
<xml_diff>
--- a/backend/uploads/Form2_EndOfTerm1_2026.xlsx
+++ b/backend/uploads/Form2_EndOfTerm1_2026.xlsx
@@ -444,28 +444,28 @@
         <v>SPP-F2-2026-006</v>
       </c>
       <c r="B2" t="str">
-        <v>Chisomo Mvula</v>
+        <v>Chikondi Mwale</v>
       </c>
       <c r="C2">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="D2">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="E2">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="F2">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="G2">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H2">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="I2">
-        <v>55</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3">
@@ -473,28 +473,28 @@
         <v>SPP-F2-2026-007</v>
       </c>
       <c r="B3" t="str">
-        <v>Innocent Chimwendo</v>
+        <v>Madalitso Tembo</v>
       </c>
       <c r="C3">
+        <v>47</v>
+      </c>
+      <c r="D3">
+        <v>54</v>
+      </c>
+      <c r="E3">
+        <v>84</v>
+      </c>
+      <c r="F3">
+        <v>90</v>
+      </c>
+      <c r="G3">
+        <v>54</v>
+      </c>
+      <c r="H3">
+        <v>66</v>
+      </c>
+      <c r="I3">
         <v>78</v>
-      </c>
-      <c r="D3">
-        <v>80</v>
-      </c>
-      <c r="E3">
-        <v>82</v>
-      </c>
-      <c r="F3">
-        <v>75</v>
-      </c>
-      <c r="G3">
-        <v>80</v>
-      </c>
-      <c r="H3">
-        <v>78</v>
-      </c>
-      <c r="I3">
-        <v>75</v>
       </c>
     </row>
     <row r="4">
@@ -502,25 +502,25 @@
         <v>SPP-F2-2026-008</v>
       </c>
       <c r="B4" t="str">
-        <v>Ruth Kalua</v>
+        <v>Mphatso Ruth Banda</v>
       </c>
       <c r="C4">
-        <v>90</v>
+        <v>54</v>
       </c>
       <c r="D4">
-        <v>88</v>
+        <v>47</v>
       </c>
       <c r="E4">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="F4">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="G4">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H4">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="I4">
         <v>90</v>
@@ -531,28 +531,28 @@
         <v>SPP-F2-2026-009</v>
       </c>
       <c r="B5" t="str">
-        <v>Patrick Nyasulu</v>
+        <v>Tadala Grace Nkhoma</v>
       </c>
       <c r="C5">
+        <v>74</v>
+      </c>
+      <c r="D5">
+        <v>42</v>
+      </c>
+      <c r="E5">
         <v>55</v>
       </c>
-      <c r="D5">
-        <v>60</v>
-      </c>
-      <c r="E5">
-        <v>58</v>
-      </c>
       <c r="F5">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="G5">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="H5">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I5">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -560,28 +560,28 @@
         <v>SPP-F2-2026-010</v>
       </c>
       <c r="B6" t="str">
-        <v>Memory Chizuma</v>
+        <v>Yamikani Chirwa</v>
       </c>
       <c r="C6">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="D6">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E6">
-        <v>75</v>
+        <v>54</v>
       </c>
       <c r="F6">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="G6">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="H6">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="I6">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add password policy, strength meter, and expanded staff types
</commit_message>
<xml_diff>
--- a/backend/uploads/Form2_EndOfTerm1_2026.xlsx
+++ b/backend/uploads/Form2_EndOfTerm1_2026.xlsx
@@ -441,10 +441,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SPP-F2-2026-006</v>
+        <v>SPP-F2-2026-001</v>
       </c>
       <c r="B2" t="str">
-        <v>Chikondi Mwale</v>
+        <v>Chisomo Mvula</v>
       </c>
       <c r="C2">
         <v>94</v>
@@ -470,10 +470,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SPP-F2-2026-007</v>
+        <v>SPP-F2-2026-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Madalitso Tembo</v>
+        <v>Innocent K Chimwendo</v>
       </c>
       <c r="C3">
         <v>47</v>
@@ -499,10 +499,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SPP-F2-2026-008</v>
+        <v>SPP-F2-2026-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Mphatso Ruth Banda</v>
+        <v>Ruth Kalua</v>
       </c>
       <c r="C4">
         <v>54</v>
@@ -528,10 +528,10 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SPP-F2-2026-009</v>
+        <v>SPP-F2-2026-004</v>
       </c>
       <c r="B5" t="str">
-        <v>Tadala Grace Nkhoma</v>
+        <v>Patrick Nyasulu</v>
       </c>
       <c r="C5">
         <v>74</v>
@@ -557,10 +557,10 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SPP-F2-2026-010</v>
+        <v>SPP-F2-2026-005</v>
       </c>
       <c r="B6" t="str">
-        <v>Yamikani Chirwa</v>
+        <v>Memory T Chizuma</v>
       </c>
       <c r="C6">
         <v>90</v>

</xml_diff>